<commit_message>
added testset and structure
</commit_message>
<xml_diff>
--- a/tests/datastructure/variable_definition_generated.xlsx
+++ b/tests/datastructure/variable_definition_generated.xlsx
@@ -431,52 +431,52 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>VaribleID</t>
+          <t>VariableName</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>VariableName</t>
+          <t>VariableDescription</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>VariableDescription</t>
+          <t>VariableUnit</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>VariableUnit</t>
+          <t>VariableType</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>VariableType</t>
+          <t>VariableDistribution</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>VariableDistribution</t>
+          <t>VariableSpreidingstype</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Spreidingstype</t>
+          <t>VariableDefaultValue</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>VariableDefaulValue</t>
+          <t>VariableLowerBound</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>VariableLowerBound</t>
+          <t>VariableUpperBound</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>VariableUpperBound</t>
+          <t>VariableMemberOf</t>
         </is>
       </c>
     </row>

</xml_diff>